<commit_message>
ADR-129, Later: No check splits into the owner answers and no check yet (backlog 0624, part 1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/StackVet - Secure by Design checklist requirements.xlsx
+++ b/exports/StackVet - Secure by Design checklist requirements.xlsx
@@ -116,7 +116,7 @@
     <t xml:space="preserve">V12.3.1 (all communications encrypted with TLS on every connection): Can be checked
 V12.3.3 (all communications between internal services encrypted with TLS): Can only be found failing
 V12.3.4 (service identity verified with trusted certificates between internal services): Can only be found failing
-V12.3.5 (service identity verified with strong authentication, such as TLS client certificates, between services): No check</t>
+V12.3.5 (service identity verified with strong authentication, such as TLS client certificates, between services): No check yet</t>
   </si>
   <si>
     <t xml:space="preserve">manual-only</t>
@@ -140,13 +140,13 @@
     <t xml:space="preserve">A central identity provider (IdP, using OIDC or OAuth2) is used, multi-factor authentication (MFA) is enforced on privileged and admin paths, and tokens are short-lived.</t>
   </si>
   <si>
-    <t xml:space="preserve">No check; a person decides</t>
+    <t xml:space="preserve">The owner answers</t>
   </si>
   <si>
     <t xml:space="preserve">A person answers it (design review); no check speaks to it</t>
   </si>
   <si>
-    <t xml:space="preserve">V6.3.3 (multi-factor authentication (MFA) enforced): No check</t>
+    <t xml:space="preserve">V6.3.3 (multi-factor authentication (MFA) enforced): The owner answers</t>
   </si>
   <si>
     <t xml:space="preserve">Decide how sign-in works and how long it lasts (design prompt, design-sign-in; trial result: shown)</t>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">V8.1.1 (access rules that apply least privilege by permissions and attributes): No check
+    <t xml:space="preserve">V8.1.1 (access rules that apply least privilege by permissions and attributes): The owner answers
 V8.2.1 (access restricted to explicit permissions, least privilege): Can be checked</t>
   </si>
   <si>
@@ -233,7 +233,7 @@
   <si>
     <t xml:space="preserve">V13.3.1 (secrets kept in a secret manager or key vault): A check helps; a person decides
 V13.3.2 (least privilege access to secrets): Can only be found failing
-V13.3.4 (secrets that expire and are rotated): No check</t>
+V13.3.4 (secrets that expire and are rotated): No check yet</t>
   </si>
   <si>
     <t xml:space="preserve">SBD-AC-06</t>
@@ -374,8 +374,8 @@
     <t xml:space="preserve">Data are classified, each class has named owners, and the controls protecting data are proportional to its classification.</t>
   </si>
   <si>
-    <t xml:space="preserve">V14.1.1 (data classified into protection levels): No check
-V14.1.2 (each data classification has documented protection controls): No check</t>
+    <t xml:space="preserve">V14.1.1 (data classified into protection levels): The owner answers
+V14.1.2 (each data classification has documented protection controls): The owner answers</t>
   </si>
   <si>
     <t xml:space="preserve">List the app's data, and keep only what it needs (design prompt, design-data-list; trial result: untested)</t>
@@ -421,7 +421,7 @@
     <t xml:space="preserve">Transactions across services use Sagas (steps that each have a compensating step to undo them), two-phase commit (2PC) is avoided, and ordinary ACID transactions within one service are preferred first.</t>
   </si>
   <si>
-    <t xml:space="preserve">V2.3.3 (transactions that either succeed entirely or are rolled back): No check</t>
+    <t xml:space="preserve">V2.3.3 (transactions that either succeed entirely or are rolled back): The owner answers</t>
   </si>
   <si>
     <t xml:space="preserve">SBD-DM-05</t>
@@ -436,8 +436,8 @@
     <t xml:space="preserve">Each class of data has retention and deletion policies, and minimization is applied, so only the data needed is collected and stored.</t>
   </si>
   <si>
-    <t xml:space="preserve">V14.1.2 (retention requirements defined for each data class): No check
-V14.2.7 (retention classification that deletes outdated data): No check</t>
+    <t xml:space="preserve">V14.1.2 (retention requirements defined for each data class): The owner answers
+V14.2.7 (retention classification that deletes outdated data): No check yet</t>
   </si>
   <si>
     <t xml:space="preserve">SBD-DM-06</t>
@@ -467,9 +467,9 @@
     <t xml:space="preserve">Logs are structured and centralized, carry correlation or trace IDs that link related entries, and administrative access is logged.</t>
   </si>
   <si>
-    <t xml:space="preserve">V16.1.1 (logs with a documented structure, formats and storage): No check
+    <t xml:space="preserve">V16.1.1 (logs with a documented structure, formats and storage): The owner answers
 V16.2.1 (log entries carrying the metadata needed to trace an event): Can be checked
-V16.4.3 (logs sent to a separate, centralized system): No check</t>
+V16.4.3 (logs sent to a separate, centralized system): The owner answers</t>
   </si>
   <si>
     <t xml:space="preserve">Decide what the app logs, and how each line reads (design prompt, design-logging; trial result: shown)</t>
@@ -629,8 +629,8 @@
     <t xml:space="preserve">All calls have timeouts, services have health probes, and critical paths have explicit failover strategies, such as running across multiple availability zones (multi-AZ).</t>
   </si>
   <si>
-    <t xml:space="preserve">V13.2.6 (timeouts and retry strategies on every connection to other services): No check
-V13.1.3 (timeouts and failure handling defined for every external service): No check</t>
+    <t xml:space="preserve">V13.2.6 (timeouts and retry strategies on every connection to other services): No check yet
+V13.1.3 (timeouts and failure handling defined for every external service): No check yet</t>
   </si>
   <si>
     <t xml:space="preserve">SBD-RR-07</t>
@@ -690,7 +690,7 @@
     <t xml:space="preserve">Where a control has ASVS counterparts, their checks are shown beside it as supporting evidence.</t>
   </si>
   <si>
-    <t xml:space="preserve">Built on 20 October 2026 from StackVet's main branch at 84d4de1b, by reading its data/ folder and tools/coverage.py.</t>
+    <t xml:space="preserve">Built on 20 October 2026 from StackVet's main branch at d6a23f2d, by reading its data/ folder and tools/coverage.py.</t>
   </si>
   <si>
     <t xml:space="preserve">Level 1</t>
@@ -2541,7 +2541,7 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
     </row>
-    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>

</xml_diff>